<commit_message>
Primeros pasos Excel DATASOURCE
</commit_message>
<xml_diff>
--- a/DATASOURCE.xlsx
+++ b/DATASOURCE.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESTUDIO\Documents\TP-IO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESTUDIO\Downloads\TP-IO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92DFE86E-E0EF-4F82-986B-C2842C1A1DBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27CE695F-9D7D-46F5-938F-C7BD5B5DD546}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13935" yWindow="0" windowWidth="13935" windowHeight="16200" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DataSource" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="40">
   <si>
     <t>DEMANDA TOTAL PAIS</t>
   </si>
@@ -102,18 +102,73 @@
     <t>DIVISION TUCUMÁN</t>
   </si>
   <si>
-    <t>NOMBRE</t>
-  </si>
-  <si>
-    <t>ALIAS</t>
+    <t>FACTOR CONVERSION</t>
+  </si>
+  <si>
+    <t>LFE</t>
+  </si>
+  <si>
+    <t>LFD</t>
+  </si>
+  <si>
+    <t>LPE</t>
+  </si>
+  <si>
+    <t>LPD</t>
+  </si>
+  <si>
+    <t>PLANTA</t>
+  </si>
+  <si>
+    <t>CAPACIDAD_LECHE_FLUIDA</t>
+  </si>
+  <si>
+    <t>CAPACIDAD_LECHE_EN_POLVO</t>
+  </si>
+  <si>
+    <t>CAPACIDAD_CREMA</t>
+  </si>
+  <si>
+    <t>CAPACIDAD_MANTECA</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>P2</t>
+  </si>
+  <si>
+    <t>P3</t>
+  </si>
+  <si>
+    <t>PARAMETRO</t>
+  </si>
+  <si>
+    <t>VALOR</t>
+  </si>
+  <si>
+    <t>LECHE_DISPONIBLE</t>
+  </si>
+  <si>
+    <t>CENTROS</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>C2</t>
+  </si>
+  <si>
+    <t>C3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="167" formatCode="0.00000"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="#,##0.000"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -229,6 +284,24 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -238,31 +311,13 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -544,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:K12"/>
+  <dimension ref="B2:K9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="28.7109375" customWidth="1"/>
@@ -558,243 +613,240 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="5"/>
-      <c r="J2" s="9" t="s">
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="13"/>
+      <c r="J2" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="10"/>
+      <c r="K2" s="15"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="F3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="H3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K3" s="12">
+      <c r="K3" s="7">
         <v>0.03</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="10" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="2">
         <v>50957</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4" s="8">
         <f>$C4 * $K$3</f>
         <v>1528.71</v>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="8">
         <f>$D4 *$K$4</f>
         <v>687.91950000000008</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="8">
         <f>$D4 *$K$5</f>
         <v>382.17750000000001</v>
       </c>
-      <c r="G4" s="13">
+      <c r="G4" s="8">
         <f>$D4 *$K$6</f>
         <v>275.1678</v>
       </c>
-      <c r="H4" s="14">
+      <c r="H4" s="9">
         <f>$D4 *$K$7</f>
         <v>183.4452</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="K4" s="12">
+      <c r="K4" s="7">
         <v>0.45</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="10" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="2">
         <v>29533</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="8">
         <f t="shared" ref="D5:D9" si="0">$C5 * $K$3</f>
         <v>885.99</v>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="8">
         <f t="shared" ref="E5:E9" si="1">D5 *$K$4</f>
         <v>398.69550000000004</v>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="8">
         <f t="shared" ref="F5:F9" si="2">$D5 *$K$5</f>
         <v>221.4975</v>
       </c>
-      <c r="G5" s="13">
+      <c r="G5" s="8">
         <f t="shared" ref="G5:G9" si="3">$D5 *$K$6</f>
         <v>159.47819999999999</v>
       </c>
-      <c r="H5" s="14">
+      <c r="H5" s="9">
         <f t="shared" ref="H5:H9" si="4">$D5 *$K$7</f>
         <v>106.3188</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="K5" s="12">
+      <c r="K5" s="7">
         <v>0.25</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="10" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="2">
         <v>2957</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="8">
         <f t="shared" si="0"/>
         <v>88.71</v>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="8">
         <f t="shared" si="1"/>
         <v>39.919499999999999</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="8">
         <f t="shared" si="2"/>
         <v>22.177499999999998</v>
       </c>
-      <c r="G6" s="13">
+      <c r="G6" s="8">
         <f t="shared" si="3"/>
         <v>15.967799999999999</v>
       </c>
-      <c r="H6" s="14">
+      <c r="H6" s="9">
         <f t="shared" si="4"/>
         <v>10.645199999999999</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="K6" s="12">
+      <c r="K6" s="7">
         <v>0.18</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="10" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="2">
         <v>1066</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="8">
         <f t="shared" si="0"/>
         <v>31.98</v>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="8">
         <f t="shared" si="1"/>
         <v>14.391</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="8">
         <f t="shared" si="2"/>
         <v>7.9950000000000001</v>
       </c>
-      <c r="G7" s="13">
+      <c r="G7" s="8">
         <f t="shared" si="3"/>
         <v>5.7564000000000002</v>
       </c>
-      <c r="H7" s="14">
+      <c r="H7" s="9">
         <f t="shared" si="4"/>
         <v>3.8376000000000001</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="K7" s="12">
+      <c r="K7" s="7">
         <v>0.12</v>
       </c>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="10" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="2">
         <v>4624</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="8">
         <f t="shared" si="0"/>
         <v>138.72</v>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="8">
         <f t="shared" si="1"/>
         <v>62.423999999999999</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="8">
         <f t="shared" si="2"/>
         <v>34.68</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="8">
         <f t="shared" si="3"/>
         <v>24.9696</v>
       </c>
-      <c r="H8" s="14">
+      <c r="H8" s="9">
         <f t="shared" si="4"/>
         <v>16.6464</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="10" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="2">
         <v>1333</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="8">
         <f t="shared" si="0"/>
         <v>39.99</v>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="8">
         <f t="shared" si="1"/>
         <v>17.9955</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="8">
         <f t="shared" si="2"/>
         <v>9.9975000000000005</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="8">
         <f t="shared" si="3"/>
         <v>7.1981999999999999</v>
       </c>
-      <c r="H9" s="14">
+      <c r="H9" s="9">
         <f t="shared" si="4"/>
         <v>4.7988</v>
       </c>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -807,15 +859,68 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CCD2DA4-F6E3-4713-B1BD-1D90C173D242}">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
         <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="16">
+        <v>1.0629999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="16">
+        <v>1.0629999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="16">
+        <v>8.7550000000000008</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="16">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="16">
+        <v>12.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="16">
+        <f>12.25/0.36</f>
+        <v>34.027777777777779</v>
       </c>
     </row>
   </sheetData>
@@ -825,18 +930,78 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7067BDC-1824-4C62-9FBC-9F18A24B1C2E}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66FF3E16-D8D9-46CF-A17E-C295F3A9DEFD}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -861,9 +1026,30 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7A8AF02-5ABE-4DD2-9200-256211114129}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2">
+        <v>24800000</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Se corrigio el modelo de LINGO, dejandolo funcional al momento de subir este commit.
</commit_message>
<xml_diff>
--- a/DATASOURCE.xlsx
+++ b/DATASOURCE.xlsx
@@ -1,14 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESTUDIO\Downloads\TP-IO\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C90C3A13-3924-4094-B58E-3A4B82A70979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="3"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SETS" sheetId="9" r:id="rId1"/>
-    <sheet name="FACTOR_CONVERSION" sheetId="3" r:id="rId2"/>
+    <sheet name="PRODUCTOS" sheetId="3" r:id="rId2"/>
     <sheet name="CAPACIDADES" sheetId="10" r:id="rId3"/>
     <sheet name="DESCREMA" sheetId="11" r:id="rId4"/>
     <sheet name="COSTOS" sheetId="12" r:id="rId5"/>
@@ -24,11 +30,12 @@
     <definedName name="COSTO" comment="Costo de mandar el Producto I desde la planta J al centro K (porfa funciona)">COSTOS!$D$2:$D$97</definedName>
     <definedName name="COSTO_LD_SF" comment="Costo de enviar leche descremada desde la planta J a la planta P3 (Santa Fe)">DESCREMA!$B$2:$B$3</definedName>
     <definedName name="DEM" comment="Demanda de producto por parte de los centros (Producto J -&gt; Centro K) (porfa funciona)">DEMANDA!$C$2:$C$33</definedName>
-    <definedName name="FACTOR_CONVERSION" comment="Factores de conversion en relacion a la leche equivalente">FACTOR_CONVERSION!$B$2:$B$9</definedName>
+    <definedName name="DESCREMA" comment="Conjunto de plantas que pueden descremar leche.">SETS!$D$2:$D$3</definedName>
+    <definedName name="FACTOR_CONVERSION" comment="Factores de conversion en relacion a la leche equivalente">PRODUCTOS!$B$2:$B$9</definedName>
     <definedName name="PLANTA" comment="Plantas que producen.">SETS!$A$2:$A$4</definedName>
     <definedName name="PRODUCTOS" comment="Productos que se producen y venden.">SETS!$C$2:$C$9</definedName>
   </definedNames>
-  <calcPr calcId="144525"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -47,7 +54,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="47">
   <si>
     <t>PRODUCTO</t>
   </si>
@@ -182,12 +189,18 @@
   </si>
   <si>
     <t>QUESO MUY BLANDO</t>
+  </si>
+  <si>
+    <t>DESCREMA</t>
+  </si>
+  <si>
+    <t>¿REFRIGERADO?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
@@ -408,7 +421,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -432,7 +445,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -443,16 +455,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -461,6 +467,8 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -734,95 +742,104 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E1" t="s">
+      <c r="D1" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="F1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D2" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" t="s">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="20" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="D3" s="21" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="20" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" t="s">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B5" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="20" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C6" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C6" s="20" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C7" t="s">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C7" s="20" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C8" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C8" s="20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="C9" t="s">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C9" s="21" t="s">
         <v>32</v>
       </c>
     </row>
@@ -833,84 +850,112 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="7">
         <v>1.0629999999999999</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>13</v>
       </c>
       <c r="B3" s="7">
         <v>1.0629999999999999</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="7">
         <v>8.7550000000000008</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>15</v>
       </c>
       <c r="B5" s="7">
         <v>12.25</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6" s="7">
         <v>12.25</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="7">
         <v>34.0277777777778</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>31</v>
       </c>
       <c r="B8" s="7">
         <v>7.2450000000000001</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>32</v>
       </c>
       <c r="B9" s="7">
         <v>2.395</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -919,8 +964,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
@@ -928,90 +973,94 @@
     <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="8">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="27">
         <v>1200000</v>
       </c>
-      <c r="C2" s="8">
+      <c r="C2" s="27">
         <v>200000</v>
       </c>
-      <c r="D2" s="8">
+      <c r="D2" s="27">
         <v>150000</v>
       </c>
-      <c r="E2" s="8">
+      <c r="E2" s="27">
         <v>70000</v>
       </c>
-      <c r="F2" s="8">
+      <c r="F2" s="28">
         <v>300000</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="8">
+      <c r="G2" s="8"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="27">
         <v>1100000</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="27">
         <v>120000</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="27">
         <v>200000</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="27">
         <v>90000</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="28">
         <v>250000</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4" s="8">
+      <c r="G3" s="8"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="27">
         <v>1350000</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="27">
         <v>110000</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="27">
         <v>0</v>
       </c>
-      <c r="E4" s="8">
+      <c r="E4" s="27">
         <v>0</v>
       </c>
-      <c r="F4" s="8">
+      <c r="F4" s="28">
         <v>250000</v>
       </c>
+      <c r="G4" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1020,8 +1069,8 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
@@ -1052,21 +1101,13 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B4">
-        <v>99999999999999</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D97"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1105,10 +1146,10 @@
       <c r="B3" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="16">
+      <c r="C3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1119,10 +1160,10 @@
       <c r="B4" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" s="16">
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1130,13 +1171,13 @@
       <c r="A5" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="19">
+      <c r="B5" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D5" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1161,10 +1202,10 @@
       <c r="B7" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="16">
+      <c r="C7" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1175,10 +1216,10 @@
       <c r="B8" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" s="16">
+      <c r="C8" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1186,13 +1227,13 @@
       <c r="A9" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D9" s="19">
+      <c r="B9" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1217,10 +1258,10 @@
       <c r="B11" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D11" s="16">
+      <c r="C11" t="s">
+        <v>26</v>
+      </c>
+      <c r="D11" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1231,10 +1272,10 @@
       <c r="B12" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" s="16">
+      <c r="C12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1242,18 +1283,18 @@
       <c r="A13" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="19">
+      <c r="B13" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D13" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="19" t="s">
         <v>13</v>
       </c>
       <c r="B14" s="12" t="s">
@@ -1267,49 +1308,49 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="21" t="s">
+      <c r="A15" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="16">
+      <c r="B15" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="15" t="s">
-        <v>21</v>
-      </c>
-      <c r="C16" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D16" s="16">
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D16" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="18" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D17" s="19">
+      <c r="B17" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D17" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="21" t="s">
+      <c r="A18" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B18" s="12" t="s">
@@ -1323,49 +1364,49 @@
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="21" t="s">
+      <c r="A19" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="16">
+      <c r="B19" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="21" t="s">
+      <c r="A20" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>22</v>
-      </c>
-      <c r="C20" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="16">
+      <c r="B20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" t="s">
+        <v>27</v>
+      </c>
+      <c r="D20" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="21" t="s">
+      <c r="A21" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="18" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D21" s="19">
+      <c r="B21" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="18">
         <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="21" t="s">
+      <c r="A22" s="20" t="s">
         <v>13</v>
       </c>
       <c r="B22" s="12" t="s">
@@ -1379,44 +1420,44 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="21" t="s">
+      <c r="A23" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C23" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="16">
+      <c r="B23" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D23" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="21" t="s">
+      <c r="A24" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="B24" s="15" t="s">
-        <v>23</v>
-      </c>
-      <c r="C24" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D24" s="16">
+      <c r="B24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D24" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D25" s="19">
+      <c r="B25" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1441,10 +1482,10 @@
       <c r="B27" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C27" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D27" s="16">
+      <c r="C27" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1455,10 +1496,10 @@
       <c r="B28" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C28" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D28" s="16">
+      <c r="C28" t="s">
+        <v>27</v>
+      </c>
+      <c r="D28" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1466,13 +1507,13 @@
       <c r="A29" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B29" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D29" s="19">
+      <c r="B29" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D29" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1497,10 +1538,10 @@
       <c r="B31" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C31" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D31" s="16">
+      <c r="C31" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1511,10 +1552,10 @@
       <c r="B32" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C32" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D32" s="16">
+      <c r="C32" t="s">
+        <v>27</v>
+      </c>
+      <c r="D32" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1522,13 +1563,13 @@
       <c r="A33" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D33" s="19">
+      <c r="B33" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D33" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1553,10 +1594,10 @@
       <c r="B35" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C35" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D35" s="16">
+      <c r="C35" t="s">
+        <v>26</v>
+      </c>
+      <c r="D35" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1567,24 +1608,24 @@
       <c r="B36" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C36" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D36" s="16">
+      <c r="C36" t="s">
+        <v>27</v>
+      </c>
+      <c r="D36" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="17" t="s">
+      <c r="A37" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B37" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C37" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D37" s="19">
+      <c r="B37" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D37" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1609,10 +1650,10 @@
       <c r="B39" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C39" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D39" s="16">
+      <c r="C39" t="s">
+        <v>26</v>
+      </c>
+      <c r="D39" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1623,10 +1664,10 @@
       <c r="B40" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C40" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D40" s="16">
+      <c r="C40" t="s">
+        <v>27</v>
+      </c>
+      <c r="D40" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1634,13 +1675,13 @@
       <c r="A41" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D41" s="19">
+      <c r="B41" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D41" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1665,10 +1706,10 @@
       <c r="B43" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C43" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D43" s="16">
+      <c r="C43" t="s">
+        <v>26</v>
+      </c>
+      <c r="D43" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1679,10 +1720,10 @@
       <c r="B44" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C44" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D44" s="16">
+      <c r="C44" t="s">
+        <v>27</v>
+      </c>
+      <c r="D44" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1690,13 +1731,13 @@
       <c r="A45" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C45" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D45" s="19">
+      <c r="B45" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C45" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D45" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1721,10 +1762,10 @@
       <c r="B47" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C47" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D47" s="16">
+      <c r="C47" t="s">
+        <v>26</v>
+      </c>
+      <c r="D47" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1735,24 +1776,24 @@
       <c r="B48" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C48" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D48" s="16">
+      <c r="C48" t="s">
+        <v>27</v>
+      </c>
+      <c r="D48" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="17" t="s">
+      <c r="A49" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B49" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C49" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D49" s="19">
+      <c r="B49" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C49" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D49" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1777,10 +1818,10 @@
       <c r="B51" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C51" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D51" s="16">
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1791,10 +1832,10 @@
       <c r="B52" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C52" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D52" s="16">
+      <c r="C52" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1802,13 +1843,13 @@
       <c r="A53" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B53" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D53" s="19">
+      <c r="B53" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D53" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1833,10 +1874,10 @@
       <c r="B55" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C55" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D55" s="16">
+      <c r="C55" t="s">
+        <v>26</v>
+      </c>
+      <c r="D55" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1847,10 +1888,10 @@
       <c r="B56" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C56" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D56" s="16">
+      <c r="C56" t="s">
+        <v>27</v>
+      </c>
+      <c r="D56" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1858,13 +1899,13 @@
       <c r="A57" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B57" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C57" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D57" s="19">
+      <c r="B57" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C57" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D57" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1889,10 +1930,10 @@
       <c r="B59" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C59" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D59" s="16">
+      <c r="C59" t="s">
+        <v>26</v>
+      </c>
+      <c r="D59" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1903,24 +1944,24 @@
       <c r="B60" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C60" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D60" s="16">
+      <c r="C60" t="s">
+        <v>27</v>
+      </c>
+      <c r="D60" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="17" t="s">
+      <c r="A61" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B61" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C61" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D61" s="19">
+      <c r="B61" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C61" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D61" s="18">
         <v>1</v>
       </c>
     </row>
@@ -1945,10 +1986,10 @@
       <c r="B63" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C63" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D63" s="16">
+      <c r="C63" t="s">
+        <v>26</v>
+      </c>
+      <c r="D63" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1959,10 +2000,10 @@
       <c r="B64" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C64" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D64" s="16">
+      <c r="C64" t="s">
+        <v>27</v>
+      </c>
+      <c r="D64" s="15">
         <v>1</v>
       </c>
     </row>
@@ -1970,13 +2011,13 @@
       <c r="A65" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B65" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C65" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D65" s="19">
+      <c r="B65" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C65" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D65" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2001,10 +2042,10 @@
       <c r="B67" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C67" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D67" s="16">
+      <c r="C67" t="s">
+        <v>26</v>
+      </c>
+      <c r="D67" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2015,10 +2056,10 @@
       <c r="B68" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C68" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D68" s="16">
+      <c r="C68" t="s">
+        <v>27</v>
+      </c>
+      <c r="D68" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2026,13 +2067,13 @@
       <c r="A69" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B69" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C69" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D69" s="19">
+      <c r="B69" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C69" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D69" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2057,10 +2098,10 @@
       <c r="B71" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C71" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D71" s="16">
+      <c r="C71" t="s">
+        <v>26</v>
+      </c>
+      <c r="D71" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2071,24 +2112,24 @@
       <c r="B72" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C72" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D72" s="16">
+      <c r="C72" t="s">
+        <v>27</v>
+      </c>
+      <c r="D72" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="17" t="s">
+      <c r="A73" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B73" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C73" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D73" s="19">
+      <c r="B73" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C73" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D73" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2113,10 +2154,10 @@
       <c r="B75" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C75" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D75" s="16">
+      <c r="C75" t="s">
+        <v>26</v>
+      </c>
+      <c r="D75" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2127,10 +2168,10 @@
       <c r="B76" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C76" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D76" s="16">
+      <c r="C76" t="s">
+        <v>27</v>
+      </c>
+      <c r="D76" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2138,13 +2179,13 @@
       <c r="A77" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B77" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C77" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D77" s="19">
+      <c r="B77" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C77" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D77" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2169,10 +2210,10 @@
       <c r="B79" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C79" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D79" s="16">
+      <c r="C79" t="s">
+        <v>26</v>
+      </c>
+      <c r="D79" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2183,10 +2224,10 @@
       <c r="B80" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C80" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D80" s="16">
+      <c r="C80" t="s">
+        <v>27</v>
+      </c>
+      <c r="D80" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2194,13 +2235,13 @@
       <c r="A81" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B81" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C81" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D81" s="19">
+      <c r="B81" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C81" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D81" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2225,10 +2266,10 @@
       <c r="B83" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C83" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D83" s="16">
+      <c r="C83" t="s">
+        <v>26</v>
+      </c>
+      <c r="D83" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2239,24 +2280,24 @@
       <c r="B84" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C84" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D84" s="16">
+      <c r="C84" t="s">
+        <v>27</v>
+      </c>
+      <c r="D84" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="17" t="s">
+      <c r="A85" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B85" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C85" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D85" s="19">
+      <c r="B85" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C85" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D85" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2281,10 +2322,10 @@
       <c r="B87" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C87" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D87" s="16">
+      <c r="C87" t="s">
+        <v>26</v>
+      </c>
+      <c r="D87" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2295,10 +2336,10 @@
       <c r="B88" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C88" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D88" s="16">
+      <c r="C88" t="s">
+        <v>27</v>
+      </c>
+      <c r="D88" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2306,13 +2347,13 @@
       <c r="A89" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B89" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C89" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D89" s="19">
+      <c r="B89" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C89" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D89" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2337,10 +2378,10 @@
       <c r="B91" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C91" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D91" s="16">
+      <c r="C91" t="s">
+        <v>26</v>
+      </c>
+      <c r="D91" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2351,10 +2392,10 @@
       <c r="B92" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C92" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D92" s="16">
+      <c r="C92" t="s">
+        <v>27</v>
+      </c>
+      <c r="D92" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2362,13 +2403,13 @@
       <c r="A93" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B93" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="C93" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D93" s="19">
+      <c r="B93" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="C93" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D93" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2393,10 +2434,10 @@
       <c r="B95" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C95" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D95" s="16">
+      <c r="C95" t="s">
+        <v>26</v>
+      </c>
+      <c r="D95" s="15">
         <v>1</v>
       </c>
     </row>
@@ -2407,24 +2448,24 @@
       <c r="B96" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="C96" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D96" s="16">
+      <c r="C96" t="s">
+        <v>27</v>
+      </c>
+      <c r="D96" s="15">
         <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="17" t="s">
+      <c r="A97" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B97" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C97" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="D97" s="19">
+      <c r="B97" s="16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C97" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="D97" s="18">
         <v>1</v>
       </c>
     </row>
@@ -2434,7 +2475,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2452,10 +2493,10 @@
       <c r="C1" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="28" t="s">
+      <c r="F1" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="29"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
@@ -2479,10 +2520,10 @@
       <c r="A3" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C3" s="16">
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="15">
         <f t="shared" ref="C3:C5" si="0">$G$9*$G$2*$G4</f>
         <v>382.17750000000001</v>
       </c>
@@ -2497,10 +2538,10 @@
       <c r="A4" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="16">
+      <c r="B4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C4" s="15">
         <f t="shared" si="0"/>
         <v>275.1678</v>
       </c>
@@ -2512,13 +2553,13 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="19">
+      <c r="B5" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="18">
         <f t="shared" si="0"/>
         <v>183.4452</v>
       </c>
@@ -2551,10 +2592,10 @@
       <c r="A7" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" s="16">
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="15">
         <f t="shared" ref="C7:C9" si="1">$G$10*$G$2*$G4</f>
         <v>221.4975</v>
       </c>
@@ -2563,10 +2604,10 @@
       <c r="A8" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C8" s="16">
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="15">
         <f t="shared" si="1"/>
         <v>159.47819999999999</v>
       </c>
@@ -2578,20 +2619,20 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C9" s="19">
+      <c r="B9" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="18">
         <f t="shared" si="1"/>
         <v>106.3188</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G9" s="23">
+      <c r="G9" s="22">
         <v>50957</v>
       </c>
     </row>
@@ -2609,7 +2650,7 @@
       <c r="F10" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="22">
         <v>29533</v>
       </c>
     </row>
@@ -2617,17 +2658,17 @@
       <c r="A11" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="16">
+      <c r="B11" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="15">
         <f t="shared" ref="C11:C13" si="2">$G$11*$G$2*$G4</f>
         <v>22.177499999999998</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="23">
+      <c r="G11" s="22">
         <v>2957</v>
       </c>
     </row>
@@ -2635,35 +2676,35 @@
       <c r="A12" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="B12" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" s="16">
+      <c r="B12" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="15">
         <f t="shared" si="2"/>
         <v>15.967799999999999</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G12" s="23">
+      <c r="G12" s="22">
         <v>1066</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C13" s="19">
+      <c r="B13" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="18">
         <f t="shared" si="2"/>
         <v>10.645199999999999</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="23">
+      <c r="G13" s="22">
         <v>4624</v>
       </c>
     </row>
@@ -2681,7 +2722,7 @@
       <c r="F14" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G14" s="23">
+      <c r="G14" s="22">
         <v>1333</v>
       </c>
     </row>
@@ -2689,17 +2730,17 @@
       <c r="A15" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C15" s="16">
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="15">
         <f t="shared" ref="C15:C17" si="3">$G$12*$G$2*$G4</f>
         <v>7.9950000000000001</v>
       </c>
-      <c r="F15" s="24" t="s">
+      <c r="F15" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="24">
         <v>0</v>
       </c>
     </row>
@@ -2707,28 +2748,28 @@
       <c r="A16" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C16" s="16">
+      <c r="B16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="15">
         <f t="shared" si="3"/>
         <v>5.7564000000000002</v>
       </c>
-      <c r="F16" s="26" t="s">
+      <c r="F16" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="27">
+      <c r="G16" s="22">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="17" t="s">
+      <c r="A17" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C17" s="19">
+      <c r="B17" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="18">
         <f t="shared" si="3"/>
         <v>3.8376000000000001</v>
       </c>
@@ -2752,10 +2793,10 @@
       <c r="A19" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B19" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C19" s="16">
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="15">
         <f t="shared" ref="C19:C21" si="4">$G$13*$G$2*$G4</f>
         <v>34.68</v>
       </c>
@@ -2764,22 +2805,22 @@
       <c r="A20" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C20" s="16">
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="15">
         <f t="shared" si="4"/>
         <v>24.9696</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C21" s="19">
+      <c r="B21" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="18">
         <f t="shared" si="4"/>
         <v>16.6464</v>
       </c>
@@ -2800,10 +2841,10 @@
       <c r="A23" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B23" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C23" s="16">
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" s="15">
         <f t="shared" ref="C23:C25" si="5">$G$14*$G$2*$G4</f>
         <v>9.9975000000000005</v>
       </c>
@@ -2812,22 +2853,22 @@
       <c r="A24" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B24" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C24" s="16">
+      <c r="B24" t="s">
+        <v>27</v>
+      </c>
+      <c r="C24" s="15">
         <f t="shared" si="5"/>
         <v>7.1981999999999999</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="17" t="s">
+      <c r="A25" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C25" s="19">
+      <c r="B25" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C25" s="18">
         <f t="shared" si="5"/>
         <v>4.7988</v>
       </c>
@@ -2848,10 +2889,10 @@
       <c r="A27" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C27" s="16">
+      <c r="B27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="15">
         <f t="shared" ref="C27:C29" si="6">$G$15*$G$2*$G4</f>
         <v>0</v>
       </c>
@@ -2860,22 +2901,22 @@
       <c r="A28" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C28" s="16">
+      <c r="B28" t="s">
+        <v>27</v>
+      </c>
+      <c r="C28" s="15">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="17" t="s">
+      <c r="A29" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C29" s="19">
+      <c r="B29" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C29" s="18">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -2896,10 +2937,10 @@
       <c r="A31" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B31" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" s="16">
+      <c r="B31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="15">
         <f t="shared" ref="C31:C33" si="7">$G$16*$G$2*$G4</f>
         <v>0</v>
       </c>
@@ -2908,22 +2949,22 @@
       <c r="A32" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B32" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="C32" s="16">
+      <c r="B32" t="s">
+        <v>27</v>
+      </c>
+      <c r="C32" s="15">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="17" t="s">
+      <c r="A33" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="C33" s="19">
+      <c r="B33" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" s="18">
         <f t="shared" si="7"/>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Modificado unas partes del DATASOURCE.xlsx. El lng quedo por algun motivo sjsj.
</commit_message>
<xml_diff>
--- a/DATASOURCE.xlsx
+++ b/DATASOURCE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ESTUDIO\Downloads\TP-IO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C90C3A13-3924-4094-B58E-3A4B82A70979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83E13F24-0676-4B8D-8BD5-02F578E9722B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="28110" windowHeight="16440" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SETS" sheetId="9" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="DESCREMA" sheetId="11" r:id="rId4"/>
     <sheet name="COSTOS" sheetId="12" r:id="rId5"/>
     <sheet name="DEMANDA" sheetId="13" r:id="rId6"/>
+    <sheet name="PARAMETROS" sheetId="14" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="CAPACIDAD_CREMA" comment="Capacidad de la planta para producir crema">CAPACIDADES!$D$2:$D$4</definedName>
@@ -32,6 +33,7 @@
     <definedName name="DEM" comment="Demanda de producto por parte de los centros (Producto J -&gt; Centro K) (porfa funciona)">DEMANDA!$C$2:$C$33</definedName>
     <definedName name="DESCREMA" comment="Conjunto de plantas que pueden descremar leche.">SETS!$D$2:$D$3</definedName>
     <definedName name="FACTOR_CONVERSION" comment="Factores de conversion en relacion a la leche equivalente">PRODUCTOS!$B$2:$B$9</definedName>
+    <definedName name="LECHE_DISPONIBLE" comment="Cantidad de materia prima disponible">PARAMETROS!$A$2</definedName>
     <definedName name="PLANTA" comment="Plantas que producen.">SETS!$A$2:$A$4</definedName>
     <definedName name="PRODUCTOS" comment="Productos que se producen y venden.">SETS!$C$2:$C$9</definedName>
   </definedNames>
@@ -54,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="65">
   <si>
     <t>PRODUCTO</t>
   </si>
@@ -195,6 +197,60 @@
   </si>
   <si>
     <t>¿REFRIGERADO?</t>
+  </si>
+  <si>
+    <t>DISTANCIA</t>
+  </si>
+  <si>
+    <t>GASTO [$/KM]</t>
+  </si>
+  <si>
+    <t>FACTOR REFRIGERADO</t>
+  </si>
+  <si>
+    <t>GASTO</t>
+  </si>
+  <si>
+    <t>Datos de otros grupos</t>
+  </si>
+  <si>
+    <t>estacionalidad leche octubre: 1,168,344,890</t>
+  </si>
+  <si>
+    <t>Ventas internas QMB: 5209.87 tn</t>
+  </si>
+  <si>
+    <t>Ventas internas QB: 16.193,30 tn</t>
+  </si>
+  <si>
+    <t>Ventas internas MT: 3698,16 tn</t>
+  </si>
+  <si>
+    <t>Ventas internas CR: 7171 * 10^3 litros</t>
+  </si>
+  <si>
+    <t>Ventas internas LPD: 1009.27 tn</t>
+  </si>
+  <si>
+    <t>Ventas internes LF: (ref) 53531, (noref) 61301 *10^3 litros</t>
+  </si>
+  <si>
+    <t>LECHE_DISPONIBLE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CABA 596.660,40 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ROS 331.477,99</t>
+  </si>
+  <si>
+    <t>MDZ 238.664,16</t>
+  </si>
+  <si>
+    <t>TUC 159.109,44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ventas LPE: </t>
   </si>
 </sst>
 </file>
@@ -204,7 +260,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -226,6 +282,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Inherit"/>
     </font>
   </fonts>
   <fills count="5">
@@ -254,7 +315,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -416,21 +477,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -443,32 +516,41 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -751,95 +833,95 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>45</v>
       </c>
       <c r="F1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:6">
+      <c r="A2" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="15" t="s">
         <v>21</v>
       </c>
       <c r="F2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="20" t="s">
+    <row r="3" spans="1:6">
+      <c r="A3" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="17" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
+    <row r="4" spans="1:6">
+      <c r="A4" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="16" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+    <row r="5" spans="1:6">
+      <c r="B5" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C6" s="20" t="s">
+    <row r="6" spans="1:6">
+      <c r="C6" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C7" s="20" t="s">
+    <row r="7" spans="1:6">
+      <c r="C7" s="16" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="20" t="s">
+    <row r="8" spans="1:6">
+      <c r="C8" s="16" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C9" s="21" t="s">
+    <row r="9" spans="1:6">
+      <c r="C9" s="17" t="s">
         <v>32</v>
       </c>
     </row>
@@ -852,14 +934,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -870,88 +952,88 @@
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="7">
+      <c r="B2" s="6">
         <v>1.0629999999999999</v>
       </c>
       <c r="C2">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <v>1.0629999999999999</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B4" s="6">
         <v>8.7550000000000008</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="6">
         <v>12.25</v>
       </c>
       <c r="C5">
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="7">
+      <c r="B6" s="6">
         <v>12.25</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="6">
         <v>34.0277777777778</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="6">
         <v>7.2450000000000001</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="7">
+      <c r="B9" s="6">
         <v>2.395</v>
       </c>
       <c r="C9">
@@ -966,7 +1048,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:I4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="25.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="28.7109375" bestFit="1" customWidth="1"/>
@@ -976,91 +1058,91 @@
     <col min="7" max="7" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>33</v>
       </c>
       <c r="I1" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="27">
+      <c r="B2" s="20">
         <v>1200000</v>
       </c>
-      <c r="C2" s="27">
+      <c r="C2" s="20">
         <v>200000</v>
       </c>
-      <c r="D2" s="27">
+      <c r="D2" s="20">
         <v>150000</v>
       </c>
-      <c r="E2" s="27">
+      <c r="E2" s="20">
         <v>70000</v>
       </c>
-      <c r="F2" s="28">
+      <c r="F2" s="21">
         <v>300000</v>
       </c>
-      <c r="G2" s="8"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:9">
       <c r="A3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="27">
+      <c r="B3" s="20">
         <v>1100000</v>
       </c>
-      <c r="C3" s="27">
+      <c r="C3" s="20">
         <v>120000</v>
       </c>
-      <c r="D3" s="27">
+      <c r="D3" s="20">
         <v>200000</v>
       </c>
-      <c r="E3" s="27">
+      <c r="E3" s="20">
         <v>90000</v>
       </c>
-      <c r="F3" s="28">
+      <c r="F3" s="21">
         <v>250000</v>
       </c>
-      <c r="G3" s="8"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:9">
       <c r="A4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="27">
+      <c r="B4" s="20">
         <v>1350000</v>
       </c>
-      <c r="C4" s="27">
+      <c r="C4" s="20">
         <v>110000</v>
       </c>
-      <c r="D4" s="27">
+      <c r="D4" s="20">
         <v>0</v>
       </c>
-      <c r="E4" s="27">
+      <c r="E4" s="20">
         <v>0</v>
       </c>
-      <c r="F4" s="28">
+      <c r="F4" s="21">
         <v>250000</v>
       </c>
-      <c r="G4" s="8"/>
+      <c r="G4" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1070,35 +1152,50 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>16</v>
       </c>
       <c r="B1" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="D1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>21</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="F2">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>22</v>
       </c>
       <c r="B3">
         <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1.05</v>
       </c>
     </row>
   </sheetData>
@@ -1108,207 +1205,309 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D97"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H97"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="6" max="6" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="20.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="9" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="G1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D2" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="D2" s="23">
+        <f>G2*H2</f>
+        <v>25372.924500000001</v>
+      </c>
+      <c r="G2" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H2" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="D3" s="18">
+        <f t="shared" ref="D3:D66" si="0">G3*H3</f>
+        <v>82609.08600000001</v>
+      </c>
+      <c r="G3" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H3" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C4" t="s">
         <v>27</v>
       </c>
-      <c r="D4" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="14" t="s">
+      <c r="D4" s="18">
+        <f t="shared" si="0"/>
+        <v>155100.6765</v>
+      </c>
+      <c r="G4" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H4" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="D5" s="19">
+        <f t="shared" si="0"/>
+        <v>174886.78200000001</v>
+      </c>
+      <c r="G5" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H5" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D6" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="D6" s="23">
+        <f t="shared" si="0"/>
+        <v>115801.17150000001</v>
+      </c>
+      <c r="G6" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H6" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C7" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="D7" s="18">
+        <f t="shared" si="0"/>
+        <v>85763.286000000007</v>
+      </c>
+      <c r="G7" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H7" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="14" t="s">
+      <c r="B8" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C8" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="14" t="s">
+      <c r="D8" s="18">
+        <f t="shared" si="0"/>
+        <v>109718.406</v>
+      </c>
+      <c r="G8" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H8" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="14" t="s">
+      <c r="D9" s="19">
+        <f t="shared" si="0"/>
+        <v>107014.90800000001</v>
+      </c>
+      <c r="G9" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H9" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="B10" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D10" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="D10" s="23">
+        <f t="shared" si="0"/>
+        <v>97121.787000000011</v>
+      </c>
+      <c r="G10" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H10" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C11" t="s">
         <v>26</v>
       </c>
-      <c r="D11" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="D11" s="18">
+        <f t="shared" si="0"/>
+        <v>48599.680500000002</v>
+      </c>
+      <c r="G11" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H11" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="14" t="s">
+      <c r="B12" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C12" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="14" t="s">
+      <c r="D12" s="18">
+        <f t="shared" si="0"/>
+        <v>136957.17000000001</v>
+      </c>
+      <c r="G12" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H12" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B13" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
+      <c r="D13" s="19">
+        <f t="shared" si="0"/>
+        <v>123569.15550000001</v>
+      </c>
+      <c r="G13" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H13" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="20" t="s">
+      <c r="D14" s="23">
+        <f t="shared" si="0"/>
+        <v>25372.924500000001</v>
+      </c>
+      <c r="G14" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H14" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B15" t="s">
@@ -1317,12 +1516,19 @@
       <c r="C15" t="s">
         <v>26</v>
       </c>
-      <c r="D15" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="20" t="s">
+      <c r="D15" s="18">
+        <f t="shared" si="0"/>
+        <v>82609.08600000001</v>
+      </c>
+      <c r="G15" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H15" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B16" t="s">
@@ -1331,40 +1537,61 @@
       <c r="C16" t="s">
         <v>27</v>
       </c>
-      <c r="D16" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="20" t="s">
+      <c r="D16" s="18">
+        <f t="shared" si="0"/>
+        <v>155100.6765</v>
+      </c>
+      <c r="G16" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H16" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="20" t="s">
+      <c r="D17" s="19">
+        <f t="shared" si="0"/>
+        <v>174886.78200000001</v>
+      </c>
+      <c r="G17" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H17" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="20" t="s">
+      <c r="D18" s="23">
+        <f t="shared" si="0"/>
+        <v>115801.17150000001</v>
+      </c>
+      <c r="G18" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H18" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B19" t="s">
@@ -1373,12 +1600,19 @@
       <c r="C19" t="s">
         <v>26</v>
       </c>
-      <c r="D19" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="20" t="s">
+      <c r="D19" s="18">
+        <f t="shared" si="0"/>
+        <v>85763.286000000007</v>
+      </c>
+      <c r="G19" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H19" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B20" t="s">
@@ -1387,40 +1621,61 @@
       <c r="C20" t="s">
         <v>27</v>
       </c>
-      <c r="D20" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="20" t="s">
+      <c r="D20" s="18">
+        <f t="shared" si="0"/>
+        <v>109718.406</v>
+      </c>
+      <c r="G20" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H20" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D21" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="20" t="s">
+      <c r="D21" s="19">
+        <f t="shared" si="0"/>
+        <v>107014.90800000001</v>
+      </c>
+      <c r="G21" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H21" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D22" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="20" t="s">
+      <c r="D22" s="23">
+        <f t="shared" si="0"/>
+        <v>97121.787000000011</v>
+      </c>
+      <c r="G22" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H22" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B23" t="s">
@@ -1429,12 +1684,19 @@
       <c r="C23" t="s">
         <v>26</v>
       </c>
-      <c r="D23" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="20" t="s">
+      <c r="D23" s="18">
+        <f t="shared" si="0"/>
+        <v>48599.680500000002</v>
+      </c>
+      <c r="G23" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H23" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" s="16" t="s">
         <v>13</v>
       </c>
       <c r="B24" t="s">
@@ -1443,1030 +1705,1548 @@
       <c r="C24" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="18">
+        <f t="shared" si="0"/>
+        <v>136957.17000000001</v>
+      </c>
+      <c r="G24" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H24" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="D25" s="19">
+        <f t="shared" si="0"/>
+        <v>123569.15550000001</v>
+      </c>
+      <c r="G25" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H25" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B26" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D26" s="23">
+        <f t="shared" si="0"/>
+        <v>24164.69</v>
+      </c>
+      <c r="G26" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H26" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="B25" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="C25" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="D25" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
+    <row r="27" spans="1:8">
+      <c r="A27" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D26" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="B27" s="14" t="s">
+      <c r="B27" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C27" t="s">
         <v>26</v>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="18">
+        <f t="shared" si="0"/>
+        <v>78675.320000000007</v>
+      </c>
+      <c r="G27" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H27" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
+    <row r="28" spans="1:8">
+      <c r="A28" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B28" s="14" t="s">
+      <c r="B28" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C28" t="s">
         <v>27</v>
       </c>
-      <c r="D28" s="15">
+      <c r="D28" s="18">
+        <f t="shared" si="0"/>
+        <v>147714.93</v>
+      </c>
+      <c r="G28" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H28" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
+    <row r="29" spans="1:8">
+      <c r="A29" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B29" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="C29" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D29" s="18">
+      <c r="D29" s="19">
+        <f t="shared" si="0"/>
+        <v>166558.84</v>
+      </c>
+      <c r="G29" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H29" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
+    <row r="30" spans="1:8">
+      <c r="A30" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B30" s="11" t="s">
+      <c r="B30" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C30" s="12" t="s">
+      <c r="C30" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D30" s="13">
+      <c r="D30" s="23">
+        <f t="shared" si="0"/>
+        <v>110286.83</v>
+      </c>
+      <c r="G30" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H30" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
+    <row r="31" spans="1:8">
+      <c r="A31" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B31" s="14" t="s">
+      <c r="B31" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C31" t="s">
         <v>26</v>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="18">
+        <f t="shared" si="0"/>
+        <v>81679.320000000007</v>
+      </c>
+      <c r="G31" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H31" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
+    <row r="32" spans="1:8">
+      <c r="A32" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B32" s="14" t="s">
+      <c r="B32" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C32" t="s">
         <v>27</v>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="18">
+        <f t="shared" si="0"/>
+        <v>104493.72</v>
+      </c>
+      <c r="G32" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H32" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
+    <row r="33" spans="1:8">
+      <c r="A33" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B33" s="16" t="s">
+      <c r="B33" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D33" s="18">
+      <c r="D33" s="19">
+        <f t="shared" si="0"/>
+        <v>101918.96</v>
+      </c>
+      <c r="G33" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H33" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
+    <row r="34" spans="1:8">
+      <c r="A34" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B34" s="11" t="s">
+      <c r="B34" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C34" s="12" t="s">
+      <c r="C34" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D34" s="13">
+      <c r="D34" s="23">
+        <f t="shared" si="0"/>
+        <v>92496.94</v>
+      </c>
+      <c r="G34" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H34" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
+    <row r="35" spans="1:8">
+      <c r="A35" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B35" s="14" t="s">
+      <c r="B35" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C35" t="s">
         <v>26</v>
       </c>
-      <c r="D35" s="15">
+      <c r="D35" s="18">
+        <f t="shared" si="0"/>
+        <v>46285.41</v>
+      </c>
+      <c r="G35" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H35" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
+    <row r="36" spans="1:8">
+      <c r="A36" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="14" t="s">
+      <c r="B36" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C36" t="s">
         <v>27</v>
       </c>
-      <c r="D36" s="15">
+      <c r="D36" s="18">
+        <f t="shared" si="0"/>
+        <v>130435.4</v>
+      </c>
+      <c r="G36" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H36" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
+    <row r="37" spans="1:8">
+      <c r="A37" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B37" s="16" t="s">
+      <c r="B37" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="C37" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D37" s="18">
+      <c r="D37" s="19">
+        <f t="shared" si="0"/>
+        <v>117684.91</v>
+      </c>
+      <c r="G37" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H37" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="11" t="s">
+    <row r="38" spans="1:8">
+      <c r="A38" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="C38" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D38" s="13">
+      <c r="D38" s="23">
+        <f t="shared" si="0"/>
+        <v>24164.69</v>
+      </c>
+      <c r="G38" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H38" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
+    <row r="39" spans="1:8">
+      <c r="A39" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="B39" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C39" t="s">
         <v>26</v>
       </c>
-      <c r="D39" s="15">
+      <c r="D39" s="18">
+        <f t="shared" si="0"/>
+        <v>78675.320000000007</v>
+      </c>
+      <c r="G39" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H39" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
+    <row r="40" spans="1:8">
+      <c r="A40" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B40" s="14" t="s">
+      <c r="B40" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C40" t="s">
         <v>27</v>
       </c>
-      <c r="D40" s="15">
+      <c r="D40" s="18">
+        <f t="shared" si="0"/>
+        <v>147714.93</v>
+      </c>
+      <c r="G40" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H40" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
+    <row r="41" spans="1:8">
+      <c r="A41" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B41" s="16" t="s">
+      <c r="B41" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="C41" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D41" s="18">
+      <c r="D41" s="19">
+        <f t="shared" si="0"/>
+        <v>166558.84</v>
+      </c>
+      <c r="G41" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H41" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
+    <row r="42" spans="1:8">
+      <c r="A42" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B42" s="11" t="s">
+      <c r="B42" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D42" s="13">
+      <c r="D42" s="23">
+        <f t="shared" si="0"/>
+        <v>110286.83</v>
+      </c>
+      <c r="G42" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H42" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
+    <row r="43" spans="1:8">
+      <c r="A43" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B43" s="14" t="s">
+      <c r="B43" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C43" t="s">
         <v>26</v>
       </c>
-      <c r="D43" s="15">
+      <c r="D43" s="18">
+        <f t="shared" si="0"/>
+        <v>81679.320000000007</v>
+      </c>
+      <c r="G43" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H43" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
+    <row r="44" spans="1:8">
+      <c r="A44" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="14" t="s">
+      <c r="B44" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C44" t="s">
         <v>27</v>
       </c>
-      <c r="D44" s="15">
+      <c r="D44" s="18">
+        <f t="shared" si="0"/>
+        <v>104493.72</v>
+      </c>
+      <c r="G44" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H44" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="14" t="s">
+    <row r="45" spans="1:8">
+      <c r="A45" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B45" s="16" t="s">
+      <c r="B45" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C45" s="17" t="s">
+      <c r="C45" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D45" s="18">
+      <c r="D45" s="19">
+        <f t="shared" si="0"/>
+        <v>101918.96</v>
+      </c>
+      <c r="G45" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H45" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="14" t="s">
+    <row r="46" spans="1:8">
+      <c r="A46" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B46" s="11" t="s">
+      <c r="B46" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C46" s="12" t="s">
+      <c r="C46" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D46" s="13">
+      <c r="D46" s="23">
+        <f t="shared" si="0"/>
+        <v>92496.94</v>
+      </c>
+      <c r="G46" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H46" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="14" t="s">
+    <row r="47" spans="1:8">
+      <c r="A47" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B47" s="14" t="s">
+      <c r="B47" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C47" t="s">
         <v>26</v>
       </c>
-      <c r="D47" s="15">
+      <c r="D47" s="18">
+        <f t="shared" si="0"/>
+        <v>46285.41</v>
+      </c>
+      <c r="G47" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H47" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="14" t="s">
+    <row r="48" spans="1:8">
+      <c r="A48" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B48" s="14" t="s">
+      <c r="B48" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C48" t="s">
         <v>27</v>
       </c>
-      <c r="D48" s="15">
+      <c r="D48" s="18">
+        <f t="shared" si="0"/>
+        <v>130435.4</v>
+      </c>
+      <c r="G48" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H48" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="16" t="s">
+    <row r="49" spans="1:8">
+      <c r="A49" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B49" s="16" t="s">
+      <c r="B49" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C49" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D49" s="18">
+      <c r="D49" s="19">
+        <f t="shared" si="0"/>
+        <v>117684.91</v>
+      </c>
+      <c r="G49" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H49" s="22">
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="11" t="s">
+    <row r="50" spans="1:8">
+      <c r="A50" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C50" s="12" t="s">
+      <c r="C50" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D50" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="14" t="s">
+      <c r="D50" s="23">
+        <f t="shared" si="0"/>
+        <v>25372.924500000001</v>
+      </c>
+      <c r="G50" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H50" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B51" s="14" t="s">
+      <c r="B51" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C51" t="s">
         <v>26</v>
       </c>
-      <c r="D51" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="14" t="s">
+      <c r="D51" s="18">
+        <f t="shared" si="0"/>
+        <v>82609.08600000001</v>
+      </c>
+      <c r="G51" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H51" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
+      <c r="A52" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B52" s="14" t="s">
+      <c r="B52" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C52" t="s">
         <v>27</v>
       </c>
-      <c r="D52" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="14" t="s">
+      <c r="D52" s="18">
+        <f t="shared" si="0"/>
+        <v>155100.6765</v>
+      </c>
+      <c r="G52" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H52" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B53" s="16" t="s">
+      <c r="B53" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C53" s="17" t="s">
+      <c r="C53" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D53" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="14" t="s">
+      <c r="D53" s="19">
+        <f t="shared" si="0"/>
+        <v>174886.78200000001</v>
+      </c>
+      <c r="G53" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H53" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B54" s="11" t="s">
+      <c r="B54" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C54" s="12" t="s">
+      <c r="C54" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D54" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="14" t="s">
+      <c r="D54" s="23">
+        <f t="shared" si="0"/>
+        <v>115801.17150000001</v>
+      </c>
+      <c r="G54" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H54" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
+      <c r="A55" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B55" s="14" t="s">
+      <c r="B55" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C55" t="s">
         <v>26</v>
       </c>
-      <c r="D55" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="14" t="s">
+      <c r="D55" s="18">
+        <f t="shared" si="0"/>
+        <v>85763.286000000007</v>
+      </c>
+      <c r="G55" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H55" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
+      <c r="A56" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B56" s="14" t="s">
+      <c r="B56" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C56" t="s">
         <v>27</v>
       </c>
-      <c r="D56" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="14" t="s">
+      <c r="D56" s="18">
+        <f t="shared" si="0"/>
+        <v>109718.406</v>
+      </c>
+      <c r="G56" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H56" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
+      <c r="A57" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B57" s="16" t="s">
+      <c r="B57" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C57" s="17" t="s">
+      <c r="C57" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D57" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="14" t="s">
+      <c r="D57" s="19">
+        <f t="shared" si="0"/>
+        <v>107014.90800000001</v>
+      </c>
+      <c r="G57" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H57" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
+      <c r="A58" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B58" s="11" t="s">
+      <c r="B58" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C58" s="12" t="s">
+      <c r="C58" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D58" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="14" t="s">
+      <c r="D58" s="23">
+        <f t="shared" si="0"/>
+        <v>97121.787000000011</v>
+      </c>
+      <c r="G58" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H58" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
+      <c r="A59" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B59" s="14" t="s">
+      <c r="B59" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C59" t="s">
         <v>26</v>
       </c>
-      <c r="D59" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="14" t="s">
+      <c r="D59" s="18">
+        <f t="shared" si="0"/>
+        <v>48599.680500000002</v>
+      </c>
+      <c r="G59" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H59" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B60" s="14" t="s">
+      <c r="B60" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C60" t="s">
         <v>27</v>
       </c>
-      <c r="D60" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="16" t="s">
+      <c r="D60" s="18">
+        <f t="shared" si="0"/>
+        <v>136957.17000000001</v>
+      </c>
+      <c r="G60" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H60" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B61" s="16" t="s">
+      <c r="B61" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C61" s="17" t="s">
+      <c r="C61" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D61" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="11" t="s">
+      <c r="D61" s="19">
+        <f t="shared" si="0"/>
+        <v>123569.15550000001</v>
+      </c>
+      <c r="G61" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H61" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B62" s="11" t="s">
+      <c r="B62" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C62" s="12" t="s">
+      <c r="C62" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D62" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="14" t="s">
+      <c r="D62" s="23">
+        <f t="shared" si="0"/>
+        <v>25372.924500000001</v>
+      </c>
+      <c r="G62" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H62" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B63" s="14" t="s">
+      <c r="B63" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C63" t="s">
         <v>26</v>
       </c>
-      <c r="D63" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="14" t="s">
+      <c r="D63" s="18">
+        <f t="shared" si="0"/>
+        <v>82609.08600000001</v>
+      </c>
+      <c r="G63" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H63" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B64" s="14" t="s">
+      <c r="B64" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C64" t="s">
         <v>27</v>
       </c>
-      <c r="D64" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="14" t="s">
+      <c r="D64" s="18">
+        <f t="shared" si="0"/>
+        <v>155100.6765</v>
+      </c>
+      <c r="G64" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H64" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B65" s="16" t="s">
+      <c r="B65" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C65" s="17" t="s">
+      <c r="C65" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D65" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="14" t="s">
+      <c r="D65" s="19">
+        <f t="shared" si="0"/>
+        <v>174886.78200000001</v>
+      </c>
+      <c r="G65" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H65" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B66" s="11" t="s">
+      <c r="B66" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C66" s="12" t="s">
+      <c r="C66" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D66" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="14" t="s">
+      <c r="D66" s="23">
+        <f t="shared" si="0"/>
+        <v>115801.17150000001</v>
+      </c>
+      <c r="G66" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H66" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B67" s="14" t="s">
+      <c r="B67" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C67" t="s">
         <v>26</v>
       </c>
-      <c r="D67" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="14" t="s">
+      <c r="D67" s="18">
+        <f t="shared" ref="D67:D97" si="1">G67*H67</f>
+        <v>85763.286000000007</v>
+      </c>
+      <c r="G67" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H67" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B68" s="14" t="s">
+      <c r="B68" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C68" t="s">
         <v>27</v>
       </c>
-      <c r="D68" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="14" t="s">
+      <c r="D68" s="18">
+        <f t="shared" si="1"/>
+        <v>109718.406</v>
+      </c>
+      <c r="G68" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H68" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B69" s="16" t="s">
+      <c r="B69" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C69" s="17" t="s">
+      <c r="C69" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D69" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="14" t="s">
+      <c r="D69" s="19">
+        <f t="shared" si="1"/>
+        <v>107014.90800000001</v>
+      </c>
+      <c r="G69" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H69" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B70" s="11" t="s">
+      <c r="B70" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C70" s="12" t="s">
+      <c r="C70" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D70" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="14" t="s">
+      <c r="D70" s="23">
+        <f t="shared" si="1"/>
+        <v>97121.787000000011</v>
+      </c>
+      <c r="G70" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H70" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
+      <c r="A71" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B71" s="14" t="s">
+      <c r="B71" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C71" t="s">
         <v>26</v>
       </c>
-      <c r="D71" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="14" t="s">
+      <c r="D71" s="18">
+        <f t="shared" si="1"/>
+        <v>48599.680500000002</v>
+      </c>
+      <c r="G71" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H71" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
+      <c r="A72" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B72" s="14" t="s">
+      <c r="B72" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C72" t="s">
         <v>27</v>
       </c>
-      <c r="D72" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="16" t="s">
+      <c r="D72" s="18">
+        <f t="shared" si="1"/>
+        <v>136957.17000000001</v>
+      </c>
+      <c r="G72" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H72" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B73" s="16" t="s">
+      <c r="B73" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C73" s="17" t="s">
+      <c r="C73" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D73" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="11" t="s">
+      <c r="D73" s="19">
+        <f t="shared" si="1"/>
+        <v>123569.15550000001</v>
+      </c>
+      <c r="G73" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H73" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B74" s="11" t="s">
+      <c r="B74" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C74" s="12" t="s">
+      <c r="C74" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D74" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="14" t="s">
+      <c r="D74" s="23">
+        <f t="shared" si="1"/>
+        <v>25372.924500000001</v>
+      </c>
+      <c r="G74" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H74" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B75" s="14" t="s">
+      <c r="B75" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C75" t="s">
         <v>26</v>
       </c>
-      <c r="D75" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="14" t="s">
+      <c r="D75" s="18">
+        <f t="shared" si="1"/>
+        <v>82609.08600000001</v>
+      </c>
+      <c r="G75" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H75" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
+      <c r="A76" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B76" s="14" t="s">
+      <c r="B76" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C76" t="s">
         <v>27</v>
       </c>
-      <c r="D76" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="14" t="s">
+      <c r="D76" s="18">
+        <f t="shared" si="1"/>
+        <v>155100.6765</v>
+      </c>
+      <c r="G76" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H76" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
+      <c r="A77" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B77" s="16" t="s">
+      <c r="B77" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C77" s="17" t="s">
+      <c r="C77" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D77" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="14" t="s">
+      <c r="D77" s="19">
+        <f t="shared" si="1"/>
+        <v>174886.78200000001</v>
+      </c>
+      <c r="G77" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H77" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
+      <c r="A78" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B78" s="11" t="s">
+      <c r="B78" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C78" s="12" t="s">
+      <c r="C78" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D78" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="14" t="s">
+      <c r="D78" s="23">
+        <f t="shared" si="1"/>
+        <v>115801.17150000001</v>
+      </c>
+      <c r="G78" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H78" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B79" s="14" t="s">
+      <c r="B79" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C79" t="s">
         <v>26</v>
       </c>
-      <c r="D79" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="14" t="s">
+      <c r="D79" s="18">
+        <f t="shared" si="1"/>
+        <v>85763.286000000007</v>
+      </c>
+      <c r="G79" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H79" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B80" s="14" t="s">
+      <c r="B80" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C80" t="s">
         <v>27</v>
       </c>
-      <c r="D80" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="14" t="s">
+      <c r="D80" s="18">
+        <f t="shared" si="1"/>
+        <v>109718.406</v>
+      </c>
+      <c r="G80" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H80" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B81" s="16" t="s">
+      <c r="B81" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C81" s="17" t="s">
+      <c r="C81" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D81" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="14" t="s">
+      <c r="D81" s="19">
+        <f t="shared" si="1"/>
+        <v>107014.90800000001</v>
+      </c>
+      <c r="G81" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H81" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="A82" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B82" s="11" t="s">
+      <c r="B82" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C82" s="12" t="s">
+      <c r="C82" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D82" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="14" t="s">
+      <c r="D82" s="23">
+        <f t="shared" si="1"/>
+        <v>97121.787000000011</v>
+      </c>
+      <c r="G82" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H82" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B83" s="14" t="s">
+      <c r="B83" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C83" t="s">
         <v>26</v>
       </c>
-      <c r="D83" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="14" t="s">
+      <c r="D83" s="18">
+        <f t="shared" si="1"/>
+        <v>48599.680500000002</v>
+      </c>
+      <c r="G83" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H83" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B84" s="14" t="s">
+      <c r="B84" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C84" t="s">
         <v>27</v>
       </c>
-      <c r="D84" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="16" t="s">
+      <c r="D84" s="18">
+        <f t="shared" si="1"/>
+        <v>136957.17000000001</v>
+      </c>
+      <c r="G84" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H84" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B85" s="16" t="s">
+      <c r="B85" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C85" s="17" t="s">
+      <c r="C85" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D85" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="11" t="s">
+      <c r="D85" s="19">
+        <f t="shared" si="1"/>
+        <v>123569.15550000001</v>
+      </c>
+      <c r="G85" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H85" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B86" s="11" t="s">
+      <c r="B86" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="C86" s="12" t="s">
+      <c r="C86" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D86" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="14" t="s">
+      <c r="D86" s="23">
+        <f t="shared" si="1"/>
+        <v>25372.924500000001</v>
+      </c>
+      <c r="G86" s="7">
+        <v>24164.69</v>
+      </c>
+      <c r="H86" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B87" s="14" t="s">
+      <c r="B87" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C87" t="s">
         <v>26</v>
       </c>
-      <c r="D87" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="14" t="s">
+      <c r="D87" s="18">
+        <f t="shared" si="1"/>
+        <v>82609.08600000001</v>
+      </c>
+      <c r="G87" s="7">
+        <v>78675.320000000007</v>
+      </c>
+      <c r="H87" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B88" s="14" t="s">
+      <c r="B88" s="12" t="s">
         <v>21</v>
       </c>
       <c r="C88" t="s">
         <v>27</v>
       </c>
-      <c r="D88" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="14" t="s">
+      <c r="D88" s="18">
+        <f t="shared" si="1"/>
+        <v>155100.6765</v>
+      </c>
+      <c r="G88" s="7">
+        <v>147714.93</v>
+      </c>
+      <c r="H88" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B89" s="16" t="s">
+      <c r="B89" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="C89" s="17" t="s">
+      <c r="C89" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D89" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="14" t="s">
+      <c r="D89" s="19">
+        <f t="shared" si="1"/>
+        <v>174886.78200000001</v>
+      </c>
+      <c r="G89" s="7">
+        <v>166558.84</v>
+      </c>
+      <c r="H89" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B90" s="11" t="s">
+      <c r="B90" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C90" s="12" t="s">
+      <c r="C90" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D90" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="14" t="s">
+      <c r="D90" s="23">
+        <f t="shared" si="1"/>
+        <v>115801.17150000001</v>
+      </c>
+      <c r="G90" s="7">
+        <v>110286.83</v>
+      </c>
+      <c r="H90" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8">
+      <c r="A91" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B91" s="14" t="s">
+      <c r="B91" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C91" t="s">
         <v>26</v>
       </c>
-      <c r="D91" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="14" t="s">
+      <c r="D91" s="18">
+        <f t="shared" si="1"/>
+        <v>85763.286000000007</v>
+      </c>
+      <c r="G91" s="7">
+        <v>81679.320000000007</v>
+      </c>
+      <c r="H91" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8">
+      <c r="A92" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B92" s="14" t="s">
+      <c r="B92" s="12" t="s">
         <v>22</v>
       </c>
       <c r="C92" t="s">
         <v>27</v>
       </c>
-      <c r="D92" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="14" t="s">
+      <c r="D92" s="18">
+        <f t="shared" si="1"/>
+        <v>109718.406</v>
+      </c>
+      <c r="G92" s="7">
+        <v>104493.72</v>
+      </c>
+      <c r="H92" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8">
+      <c r="A93" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B93" s="16" t="s">
+      <c r="B93" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="C93" s="17" t="s">
+      <c r="C93" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D93" s="18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="14" t="s">
+      <c r="D93" s="19">
+        <f t="shared" si="1"/>
+        <v>107014.90800000001</v>
+      </c>
+      <c r="G93" s="7">
+        <v>101918.96</v>
+      </c>
+      <c r="H93" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8">
+      <c r="A94" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B94" s="11" t="s">
+      <c r="B94" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C94" s="12" t="s">
+      <c r="C94" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="D94" s="13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="14" t="s">
+      <c r="D94" s="23">
+        <f t="shared" si="1"/>
+        <v>97121.787000000011</v>
+      </c>
+      <c r="G94" s="7">
+        <v>92496.94</v>
+      </c>
+      <c r="H94" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8">
+      <c r="A95" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B95" s="14" t="s">
+      <c r="B95" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C95" t="s">
         <v>26</v>
       </c>
-      <c r="D95" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="14" t="s">
+      <c r="D95" s="18">
+        <f t="shared" si="1"/>
+        <v>48599.680500000002</v>
+      </c>
+      <c r="G95" s="7">
+        <v>46285.41</v>
+      </c>
+      <c r="H95" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8">
+      <c r="A96" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B96" s="14" t="s">
+      <c r="B96" s="12" t="s">
         <v>23</v>
       </c>
       <c r="C96" t="s">
         <v>27</v>
       </c>
-      <c r="D96" s="15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="16" t="s">
+      <c r="D96" s="18">
+        <f t="shared" si="1"/>
+        <v>136957.17000000001</v>
+      </c>
+      <c r="G96" s="7">
+        <v>130435.4</v>
+      </c>
+      <c r="H96" s="22">
+        <v>1.05</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8">
+      <c r="A97" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B97" s="16" t="s">
+      <c r="B97" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="C97" s="17" t="s">
+      <c r="C97" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="D97" s="18">
-        <v>1</v>
+      <c r="D97" s="19">
+        <f t="shared" si="1"/>
+        <v>123569.15550000001</v>
+      </c>
+      <c r="G97" s="7">
+        <v>117684.91</v>
+      </c>
+      <c r="H97" s="22">
+        <v>1.05</v>
       </c>
     </row>
   </sheetData>
@@ -2476,38 +3256,38 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
-    <col min="6" max="6" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.28515625" customWidth="1"/>
     <col min="7" max="7" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="C1" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F1" s="25" t="s">
+      <c r="F1" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="G1" s="26"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="G1" s="25"/>
+    </row>
+    <row r="2" spans="1:11">
+      <c r="A2" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="13">
+      <c r="C2" s="23">
         <f>$G$9*$G$2*$G3</f>
-        <v>687.91950000000008</v>
+        <v>546191.91</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>7</v>
@@ -2515,17 +3295,20 @@
       <c r="G2" s="3">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="14" t="s">
+      <c r="K2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
+      <c r="A3" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B3" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="15">
-        <f t="shared" ref="C3:C5" si="0">$G$9*$G$2*$G4</f>
-        <v>382.17750000000001</v>
+      <c r="C3" s="18">
+        <f>$G$9*$G$2*$G4</f>
+        <v>303439.95</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>8</v>
@@ -2533,17 +3316,20 @@
       <c r="G3" s="3">
         <v>0.45</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="14" t="s">
+      <c r="K3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" s="12" t="s">
         <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="15">
-        <f t="shared" si="0"/>
-        <v>275.1678</v>
+      <c r="C4" s="18">
+        <f>$G$9*$G$2*$G5</f>
+        <v>218476.764</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>9</v>
@@ -2551,17 +3337,20 @@
       <c r="G4" s="3">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="K4" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="18">
-        <f t="shared" si="0"/>
-        <v>183.4452</v>
+      <c r="C5" s="19">
+        <f>$G$9*$G$2*$G6</f>
+        <v>145651.17600000001</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>10</v>
@@ -2569,17 +3358,20 @@
       <c r="G5" s="3">
         <v>0.18</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+      <c r="K5" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
+      <c r="A6" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="23">
         <f>$G$10*$G$2*$G3</f>
-        <v>398.69550000000004</v>
+        <v>281371.58999999997</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>11</v>
@@ -2587,386 +3379,419 @@
       <c r="G6" s="3">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="K6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B7" t="s">
         <v>26</v>
       </c>
-      <c r="C7" s="15">
-        <f t="shared" ref="C7:C9" si="1">$G$10*$G$2*$G4</f>
-        <v>221.4975</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="14" t="s">
+      <c r="C7" s="18">
+        <f>$G$10*$G$2*$G4</f>
+        <v>156317.54999999999</v>
+      </c>
+      <c r="K7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
+      <c r="A8" s="12" t="s">
         <v>13</v>
       </c>
       <c r="B8" t="s">
         <v>27</v>
       </c>
-      <c r="C8" s="15">
-        <f t="shared" si="1"/>
-        <v>159.47819999999999</v>
-      </c>
-      <c r="F8" s="5" t="s">
+      <c r="C8" s="18">
+        <f>$G$10*$G$2*$G5</f>
+        <v>112548.63599999998</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="5" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="K8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
+      <c r="A9" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="18">
-        <f t="shared" si="1"/>
-        <v>106.3188</v>
-      </c>
-      <c r="F9" s="4" t="s">
+      <c r="C9" s="19">
+        <f>$G$10*$G$2*$G6</f>
+        <v>75032.423999999985</v>
+      </c>
+      <c r="F9" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="G9" s="22">
-        <v>50957</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+      <c r="G9" s="28">
+        <v>40458660</v>
+      </c>
+      <c r="I9" s="32">
+        <v>40458660</v>
+      </c>
+      <c r="K9" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
+      <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="23">
         <f>$G$11*$G$2*$G3</f>
-        <v>39.919499999999999</v>
-      </c>
-      <c r="F10" s="4" t="s">
+        <v>39919.5</v>
+      </c>
+      <c r="F10" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="G10" s="22">
-        <v>29533</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="G10" s="28">
+        <v>20842340</v>
+      </c>
+      <c r="I10" s="32">
+        <v>20842340</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
+      <c r="A11" s="12" t="s">
         <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="15">
-        <f t="shared" ref="C11:C13" si="2">$G$11*$G$2*$G4</f>
-        <v>22.177499999999998</v>
-      </c>
-      <c r="F11" s="4" t="s">
+      <c r="C11" s="18">
+        <f t="shared" ref="C11:C13" si="0">$G$11*$G$2*$G4</f>
+        <v>22177.5</v>
+      </c>
+      <c r="F11" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="G11" s="22">
-        <v>2957</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="14" t="s">
+      <c r="G11" s="28">
+        <v>2957000</v>
+      </c>
+      <c r="K11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="30">
+      <c r="A12" s="12" t="s">
         <v>14</v>
       </c>
       <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="15">
-        <f t="shared" si="2"/>
-        <v>15.967799999999999</v>
-      </c>
-      <c r="F12" s="4" t="s">
+      <c r="C12" s="18">
+        <f t="shared" si="0"/>
+        <v>15967.8</v>
+      </c>
+      <c r="F12" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="G12" s="22">
-        <v>1066</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+      <c r="G12" s="28">
+        <v>1009270</v>
+      </c>
+      <c r="K12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
+      <c r="A13" s="13" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="18">
-        <f t="shared" si="2"/>
-        <v>10.645199999999999</v>
-      </c>
-      <c r="F13" s="4" t="s">
+      <c r="C13" s="19">
+        <f t="shared" si="0"/>
+        <v>10645.199999999999</v>
+      </c>
+      <c r="F13" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="G13" s="22">
-        <v>4624</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
+      <c r="G13" s="28">
+        <v>7171000</v>
+      </c>
+      <c r="K13" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
+      <c r="A14" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="12" t="s">
+      <c r="B14" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="13">
+      <c r="C14" s="23">
         <f>$G$12*$G$2*$G3</f>
-        <v>14.391</v>
-      </c>
-      <c r="F14" s="4" t="s">
+        <v>13625.145</v>
+      </c>
+      <c r="F14" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="G14" s="22">
-        <v>1333</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="14" t="s">
+      <c r="G14" s="28">
+        <v>1333000</v>
+      </c>
+      <c r="K14" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
+      <c r="A15" s="12" t="s">
         <v>15</v>
       </c>
       <c r="B15" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="15">
-        <f t="shared" ref="C15:C17" si="3">$G$12*$G$2*$G4</f>
-        <v>7.9950000000000001</v>
-      </c>
-      <c r="F15" s="23" t="s">
+      <c r="C15" s="18">
+        <f t="shared" ref="C15:C17" si="1">$G$12*$G$2*$G4</f>
+        <v>7569.5249999999996</v>
+      </c>
+      <c r="F15" s="31" t="s">
         <v>43</v>
       </c>
-      <c r="G15" s="24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="14" t="s">
+      <c r="G15" s="29">
+        <v>16193300</v>
+      </c>
+      <c r="K15" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
+      <c r="A16" s="12" t="s">
         <v>15</v>
       </c>
       <c r="B16" t="s">
         <v>27</v>
       </c>
-      <c r="C16" s="15">
-        <f t="shared" si="3"/>
-        <v>5.7564000000000002</v>
-      </c>
-      <c r="F16" s="4" t="s">
+      <c r="C16" s="18">
+        <f t="shared" si="1"/>
+        <v>5450.0579999999991</v>
+      </c>
+      <c r="F16" s="30" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="G16" s="28">
+        <v>5209870</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C17" s="18">
-        <f t="shared" si="3"/>
-        <v>3.8376000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
+      <c r="C17" s="19">
+        <f t="shared" si="1"/>
+        <v>3633.3719999999998</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="23">
         <f>$G$13*$G$2*$G3</f>
-        <v>62.423999999999999</v>
+        <v>96808.5</v>
       </c>
       <c r="F18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="14" t="s">
+    <row r="19" spans="1:6">
+      <c r="A19" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="15">
-        <f t="shared" ref="C19:C21" si="4">$G$13*$G$2*$G4</f>
-        <v>34.68</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
+      <c r="C19" s="18">
+        <f t="shared" ref="C19:C21" si="2">$G$13*$G$2*$G4</f>
+        <v>53782.5</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B20" t="s">
         <v>27</v>
       </c>
-      <c r="C20" s="15">
-        <f t="shared" si="4"/>
-        <v>24.9696</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="C20" s="18">
+        <f t="shared" si="2"/>
+        <v>38723.4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="18">
-        <f t="shared" si="4"/>
-        <v>16.6464</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
+      <c r="C21" s="19">
+        <f t="shared" si="2"/>
+        <v>25815.599999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="12" t="s">
+      <c r="B22" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="13">
+      <c r="C22" s="23">
         <f>$G$14*$G$2*$G3</f>
-        <v>17.9955</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
+        <v>17995.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B23" t="s">
         <v>26</v>
       </c>
-      <c r="C23" s="15">
-        <f t="shared" ref="C23:C25" si="5">$G$14*$G$2*$G4</f>
-        <v>9.9975000000000005</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
+      <c r="C23" s="18">
+        <f t="shared" ref="C23:C25" si="3">$G$14*$G$2*$G4</f>
+        <v>9997.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B24" t="s">
         <v>27</v>
       </c>
-      <c r="C24" s="15">
-        <f t="shared" si="5"/>
-        <v>7.1981999999999999</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
+      <c r="C24" s="18">
+        <f t="shared" si="3"/>
+        <v>7198.2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6">
+      <c r="A25" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C25" s="18">
-        <f t="shared" si="5"/>
-        <v>4.7988</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
+      <c r="C25" s="19">
+        <f t="shared" si="3"/>
+        <v>4798.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6">
+      <c r="A26" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="12" t="s">
+      <c r="B26" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="13">
+      <c r="C26" s="23">
         <f>$G$15*$G$2*$G3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
+        <v>218609.55000000002</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="12" t="s">
         <v>31</v>
       </c>
       <c r="B27" t="s">
         <v>26</v>
       </c>
-      <c r="C27" s="15">
-        <f t="shared" ref="C27:C29" si="6">$G$15*$G$2*$G4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
+      <c r="C27" s="18">
+        <f t="shared" ref="C27:C29" si="4">$G$15*$G$2*$G4</f>
+        <v>121449.75</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="12" t="s">
         <v>31</v>
       </c>
       <c r="B28" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="15">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
+      <c r="C28" s="18">
+        <f t="shared" si="4"/>
+        <v>87443.819999999992</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6">
+      <c r="A29" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="B29" s="17" t="s">
+      <c r="B29" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="18">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
+      <c r="C29" s="19">
+        <f t="shared" si="4"/>
+        <v>58295.88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6">
+      <c r="A30" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B30" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C30" s="13">
+      <c r="C30" s="23">
         <f>$G$16*$G$2*$G3</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
+        <v>70333.24500000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6">
+      <c r="A31" s="12" t="s">
         <v>32</v>
       </c>
       <c r="B31" t="s">
         <v>26</v>
       </c>
-      <c r="C31" s="15">
-        <f t="shared" ref="C31:C33" si="7">$G$16*$G$2*$G4</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
+      <c r="C31" s="18">
+        <f t="shared" ref="C31:C33" si="5">$G$16*$G$2*$G4</f>
+        <v>39074.025000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6">
+      <c r="A32" s="12" t="s">
         <v>32</v>
       </c>
       <c r="B32" t="s">
         <v>27</v>
       </c>
-      <c r="C32" s="15">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
+      <c r="C32" s="18">
+        <f t="shared" si="5"/>
+        <v>28133.297999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="17" t="s">
+      <c r="B33" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="18">
-        <f t="shared" si="7"/>
-        <v>0</v>
+      <c r="C33" s="19">
+        <f t="shared" si="5"/>
+        <v>18755.531999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2975,4 +3800,27 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44F2F6F6-1337-4953-8B5F-A60C64F6CF43}">
+  <dimension ref="A1:A2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="26" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="27">
+        <v>1168344890</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>